<commit_message>
vist töötab,aga peab testima
</commit_message>
<xml_diff>
--- a/firmad.xlsx
+++ b/firmad.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proge\Python\Rannahall\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proge_(laptop)\Python\Rannahall\autom-meilide-saatm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F02559A-69DD-47B9-8A65-C76EF854D6EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04561E94-916D-49E9-931E-818177931EC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1965" windowWidth="24915" windowHeight="13605" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Leht1" sheetId="1" r:id="rId1"/>
@@ -25,31 +25,25 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
-    <t>LÄHEDAL ASUVAD FIRMAD</t>
+    <t>FIRMA</t>
   </si>
   <si>
-    <t>Meil</t>
-  </si>
-  <si>
-    <t>Marienthali keskus</t>
-  </si>
-  <si>
-    <t>Marienthali keskuse KÕRVAL</t>
+    <t>E-POST</t>
   </si>
   <si>
     <t>sverkersaar@gmail.com</t>
   </si>
   <si>
-    <t>Triip</t>
+    <t>Mark OÜ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -58,25 +52,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="186"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="16"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="186"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="186"/>
     </font>
@@ -89,7 +75,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -98,18 +84,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA4C2F4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
+        <fgColor rgb="FFD9E2F3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -132,64 +112,23 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hüperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="3">
+    <cellStyle name="Hüperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normaallaad" xfId="0" builtinId="0"/>
+    <cellStyle name="Normaallaad 2" xfId="1" xr:uid="{AE6A0AD6-ABF9-47A5-B0DF-42A16EDA9B94}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -210,13 +149,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>1</xdr:row>
       <xdr:rowOff>9525</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -533,49 +472,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="54" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:2" ht="42.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
     </row>
-    <row r="2" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2"/>
-    </row>
-    <row r="3" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="7"/>
-    </row>
-    <row r="4" spans="1:2" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>5</v>
+      <c r="B2" t="s">
+        <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="7"/>
-    </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A5:B5"/>
-  </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A4" r:id="rId1" xr:uid="{32C5CDC8-95F5-4545-ADC9-563B50062C60}"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{16CEC700-E155-4BEA-9115-8DF3563FDA10}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>

</xml_diff>